<commit_message>
Stage 8 review fixes: B-030
</commit_message>
<xml_diff>
--- a/output/archive/BrindlewytheData/Studies/2025/BW25_0486/Tracking/BW25_0486_screen_gate_tracker.xlsx
+++ b/output/archive/BrindlewytheData/Studies/2025/BW25_0486/Tracking/BW25_0486_screen_gate_tracker.xlsx
@@ -175,7 +175,7 @@
     </comment>
     <comment ref="E14" authorId="1" shapeId="0">
       <text>
-        <t>TODO: plate 4 allocation is still missing. Stéphane to confirm before anyone signs the readout.</t>
+        <t>TODO: reconcile plate allocation against the original run sheets before anyone signs the readout.</t>
       </text>
     </comment>
   </commentList>
@@ -190,7 +190,7 @@
   <commentList>
     <comment ref="A2" authorId="0" shapeId="0">
       <text>
-        <t>Benchmark counts the full set, these rows do not. Keep both until the readout is signed off.</t>
+        <t>FM20-02108 records a cell exclusion for low seal resistance. Keep that qualification and reconcile any repeat action with the original run sheets; this tracker remains unfinished.</t>
       </text>
     </comment>
   </commentList>
@@ -499,7 +499,8 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>FM20 hERG screen: screen gate tracker</t>
+          <t>Brindlewythe Biosciences Ltd, a Tarnovell company
+FM20 hERG screen: screen gate tracker</t>
         </is>
       </c>
     </row>
@@ -569,7 +570,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>On hold since 15/12/2025. Paused while the nomination committee reviews a new efficacy concern. Not related to the assay.</t>
+          <t>On hold at 15/12/2025. Farnovessa paused the screen while its nomination committee reviews a new efficacy concern unrelated to the assay.</t>
         </is>
       </c>
     </row>
@@ -786,43 +787,23 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Shipment 1</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>19/11/2025</t>
-        </is>
-      </c>
+          <t>Original shipment record</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr"/>
       <c r="C3" s="2" t="inlineStr"/>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Intact</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Henning Flantz</t>
-        </is>
-      </c>
+      <c r="D3" s="2" t="inlineStr"/>
+      <c r="E3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Shipment 2</t>
-        </is>
-      </c>
+      <c r="A4" s="2" t="inlineStr"/>
       <c r="B4" s="2" t="inlineStr"/>
       <c r="C4" s="2" t="inlineStr"/>
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Shipment 3</t>
-        </is>
-      </c>
+      <c r="A5" s="2" t="inlineStr"/>
       <c r="B5" s="2" t="inlineStr"/>
       <c r="C5" s="2" t="inlineStr"/>
       <c r="D5" s="2" t="inlineStr"/>
@@ -832,7 +813,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Count each shipment against the sample card list before release to plates.</t>
+          <t>TODO: reconcile shipment receipt against the original sample cards; receipt fields remain unfinished.</t>
         </is>
       </c>
     </row>
@@ -895,74 +876,34 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>FM20-02000 to FM20-02010</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Jason Scanlon</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>25/11/2025</t>
-        </is>
-      </c>
+          <t>Original plate allocation record</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr"/>
+      <c r="C3" s="2" t="inlineStr"/>
+      <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>TODO</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>FM20-02012 to FM20-02018</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Jason Scanlon</t>
-        </is>
-      </c>
+      <c r="A4" s="2" t="inlineStr"/>
+      <c r="B4" s="2" t="inlineStr"/>
+      <c r="C4" s="2" t="inlineStr"/>
       <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
+      <c r="E4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
+      <c r="A5" s="2" t="inlineStr"/>
       <c r="B5" s="2" t="inlineStr"/>
       <c r="C5" s="2" t="inlineStr"/>
       <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
+      <c r="E5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
+      <c r="A6" s="2" t="inlineStr"/>
       <c r="B6" s="2" t="inlineStr"/>
       <c r="C6" s="2" t="inlineStr"/>
       <c r="D6" s="2" t="inlineStr"/>
@@ -1003,7 +944,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>The remaining compounds were not read before the pause. TODO: reconcile this sheet with the benchmark before anyone quotes a figure.</t>
+          <t>Partial data only; work stopped. TODO: reconcile outstanding records and QC follow-up before release. Project benchmark counts describe the full screening set and must not be treated as counts of these displayed rows.</t>
         </is>
       </c>
     </row>

</xml_diff>